<commit_message>
chore(data): add security event to map config + update compliance matrix
- map_config.json：新增暴力事件（EV-0425-001）至指揮部地圖
- ICS_DMAS_master_capability_matrix.xlsx：HOTFIX-WS-01 close 後
  CAP-013 Status / Evidence 欄位更新（Step C C-3）

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/compliance/ICS_DMAS_master_capability_matrix.xlsx
+++ b/docs/compliance/ICS_DMAS_master_capability_matrix.xlsx
@@ -5,10 +5,10 @@
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/dd2d3534488626a3/文件/民防/研究資料/! [研究] ICS_DMAS_docs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yello\研究計畫\ICS_DMAS\docs\compliance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="11_FF57A87D6457DD570D45840AA31CCED1EFE1B979" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9E5C41CC-025B-422A-99C6-0C14335D7F1B}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57CF6AFC-5703-4BF1-9938-27C67464CD41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="843" uniqueCount="564">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="844" uniqueCount="565">
   <si>
     <t>ICS_DMAS Master Capability Matrix</t>
   </si>
@@ -692,9 +692,6 @@
   </si>
   <si>
     <t>不建議外部宣稱細節</t>
-  </si>
-  <si>
-    <t>Needs Hotfix</t>
   </si>
   <si>
     <t>列為 HOTFIX-WS-01</t>
@@ -1853,12 +1850,37 @@
     </r>
     <phoneticPr fontId="8" type="noConversion"/>
   </si>
+  <si>
+    <t>Last Update</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="10"/>
+        <color rgb="FF111827"/>
+        <rFont val="Carlito"/>
+        <family val="2"/>
+      </rPr>
+      <t>Needs Hotfix</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF111827"/>
+        <rFont val="Carlito"/>
+      </rPr>
+      <t xml:space="preserve"> -&gt; Partial Hardened</t>
+    </r>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -1946,6 +1968,11 @@
       <family val="2"/>
       <charset val="136"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Carlito"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -1956,7 +1983,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
+        <fgColor theme="9" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1983,7 +2010,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
@@ -1991,10 +2018,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -2011,6 +2034,12 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
@@ -2055,8 +2084,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="CapabilityMatrix" displayName="CapabilityMatrix" ref="A4:T38">
-  <tableColumns count="20">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="CapabilityMatrix" displayName="CapabilityMatrix" ref="A4:U38">
+  <tableColumns count="21">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Capability ID"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Capability"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="Capability Group"/>
@@ -2077,6 +2106,7 @@
     <tableColumn id="18" xr3:uid="{00000000-0010-0000-0200-000012000000}" name="Owner"/>
     <tableColumn id="19" xr3:uid="{00000000-0010-0000-0200-000013000000}" name="Priority"/>
     <tableColumn id="20" xr3:uid="{00000000-0010-0000-0200-000014000000}" name="Disclosure"/>
+    <tableColumn id="21" xr3:uid="{AFEB0359-48C2-466B-8D9A-13AD724F7F93}" name="Last Update"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2289,18 +2319,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="27.9" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
       <c r="K1" s="4"/>
       <c r="L1" s="4"/>
       <c r="M1" s="4"/>
@@ -2319,18 +2349,18 @@
       <c r="Z1" s="4"/>
     </row>
     <row r="2" spans="1:26" ht="33.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
-      <c r="I2" s="10"/>
-      <c r="J2" s="10"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
+      <c r="J2" s="18"/>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
@@ -2455,11 +2485,12 @@
     <col min="13" max="13" width="22" customWidth="1"/>
     <col min="14" max="14" width="45" customWidth="1"/>
     <col min="15" max="15" width="36" customWidth="1"/>
-    <col min="16" max="16" width="18" style="12" customWidth="1"/>
+    <col min="16" max="16" width="16.77734375" style="8" customWidth="1"/>
     <col min="17" max="17" width="42" customWidth="1"/>
     <col min="18" max="18" width="22" customWidth="1"/>
     <col min="19" max="19" width="10" customWidth="1"/>
     <col min="20" max="20" width="22" customWidth="1"/>
+    <col min="21" max="21" width="13.88671875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="27.9" customHeight="1" x14ac:dyDescent="0.4">
@@ -2480,7 +2511,7 @@
       <c r="M1" s="4"/>
       <c r="N1" s="4"/>
       <c r="O1" s="4"/>
-      <c r="P1" s="11"/>
+      <c r="P1" s="7"/>
       <c r="Q1" s="4"/>
       <c r="R1" s="4"/>
       <c r="S1" s="4"/>
@@ -2543,7 +2574,7 @@
       <c r="O4" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="P4" s="13" t="s">
+      <c r="P4" s="9" t="s">
         <v>38</v>
       </c>
       <c r="Q4" s="1" t="s">
@@ -2557,6 +2588,9 @@
       </c>
       <c r="T4" s="1" t="s">
         <v>42</v>
+      </c>
+      <c r="U4" s="13" t="s">
+        <v>563</v>
       </c>
     </row>
     <row r="5" spans="1:26" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
@@ -2605,7 +2639,7 @@
       <c r="O5" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="P5" s="14" t="s">
+      <c r="P5" s="10" t="s">
         <v>58</v>
       </c>
       <c r="Q5" s="3" t="s">
@@ -2667,7 +2701,7 @@
       <c r="O6" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="P6" s="14" t="s">
+      <c r="P6" s="10" t="s">
         <v>58</v>
       </c>
       <c r="Q6" s="3" t="s">
@@ -2729,7 +2763,7 @@
       <c r="O7" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="P7" s="14" t="s">
+      <c r="P7" s="10" t="s">
         <v>58</v>
       </c>
       <c r="Q7" s="3" t="s">
@@ -2791,7 +2825,7 @@
       <c r="O8" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="P8" s="14" t="s">
+      <c r="P8" s="10" t="s">
         <v>58</v>
       </c>
       <c r="Q8" s="3" t="s">
@@ -2853,7 +2887,7 @@
       <c r="O9" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="P9" s="14" t="s">
+      <c r="P9" s="10" t="s">
         <v>58</v>
       </c>
       <c r="Q9" s="3" t="s">
@@ -2915,7 +2949,7 @@
       <c r="O10" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="P10" s="14" t="s">
+      <c r="P10" s="10" t="s">
         <v>17</v>
       </c>
       <c r="Q10" s="3" t="s">
@@ -2977,7 +3011,7 @@
       <c r="O11" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="P11" s="14" t="s">
+      <c r="P11" s="10" t="s">
         <v>17</v>
       </c>
       <c r="Q11" s="3" t="s">
@@ -3039,7 +3073,7 @@
       <c r="O12" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="P12" s="14" t="s">
+      <c r="P12" s="10" t="s">
         <v>58</v>
       </c>
       <c r="Q12" s="3" t="s">
@@ -3101,7 +3135,7 @@
       <c r="O13" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="P13" s="14" t="s">
+      <c r="P13" s="10" t="s">
         <v>17</v>
       </c>
       <c r="Q13" s="3" t="s">
@@ -3118,7 +3152,7 @@
       </c>
     </row>
     <row r="14" spans="1:26" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="17" t="s">
+      <c r="A14" s="19" t="s">
         <v>168</v>
       </c>
       <c r="B14" s="3" t="s">
@@ -3163,11 +3197,11 @@
       <c r="O14" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="P14" s="15" t="s">
+      <c r="P14" s="11" t="s">
+        <v>561</v>
+      </c>
+      <c r="Q14" s="12" t="s">
         <v>562</v>
-      </c>
-      <c r="Q14" s="16" t="s">
-        <v>563</v>
       </c>
       <c r="R14" s="3" t="s">
         <v>180</v>
@@ -3177,6 +3211,9 @@
       </c>
       <c r="T14" s="3" t="s">
         <v>181</v>
+      </c>
+      <c r="U14" s="14">
+        <v>46138</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
@@ -3225,7 +3262,7 @@
       <c r="O15" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="P15" s="14" t="s">
+      <c r="P15" s="10" t="s">
         <v>58</v>
       </c>
       <c r="Q15" s="3" t="s">
@@ -3287,7 +3324,7 @@
       <c r="O16" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="P16" s="14" t="s">
+      <c r="P16" s="10" t="s">
         <v>17</v>
       </c>
       <c r="Q16" s="3" t="s">
@@ -3303,8 +3340,8 @@
         <v>181</v>
       </c>
     </row>
-    <row r="17" spans="1:20" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="3" t="s">
+    <row r="17" spans="1:21" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="19" t="s">
         <v>207</v>
       </c>
       <c r="B17" s="3" t="s">
@@ -3349,14 +3386,14 @@
       <c r="O17" s="3" t="s">
         <v>216</v>
       </c>
-      <c r="P17" s="14" t="s">
+      <c r="P17" s="11" t="s">
+        <v>564</v>
+      </c>
+      <c r="Q17" s="3" t="s">
         <v>217</v>
       </c>
-      <c r="Q17" s="3" t="s">
+      <c r="R17" s="3" t="s">
         <v>218</v>
-      </c>
-      <c r="R17" s="3" t="s">
-        <v>219</v>
       </c>
       <c r="S17" s="3" t="s">
         <v>77</v>
@@ -3364,25 +3401,28 @@
       <c r="T17" s="3" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="18" spans="1:20" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="U17" s="14">
+        <v>46138</v>
+      </c>
+    </row>
+    <row r="18" spans="1:21" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="B18" s="3" t="s">
         <v>220</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="C18" s="3" t="s">
         <v>221</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="D18" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="E18" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="E18" s="3" t="s">
+      <c r="F18" s="3" t="s">
         <v>224</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>225</v>
       </c>
       <c r="G18" s="3" t="s">
         <v>49</v>
@@ -3391,34 +3431,34 @@
         <v>67</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="J18" s="3" t="s">
         <v>124</v>
       </c>
       <c r="K18" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="L18" s="3" t="s">
         <v>227</v>
-      </c>
-      <c r="L18" s="3" t="s">
-        <v>228</v>
       </c>
       <c r="M18" s="3" t="s">
         <v>164</v>
       </c>
       <c r="N18" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="O18" s="3" t="s">
         <v>229</v>
       </c>
-      <c r="O18" s="3" t="s">
+      <c r="P18" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q18" s="3" t="s">
         <v>230</v>
       </c>
-      <c r="P18" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q18" s="3" t="s">
+      <c r="R18" s="3" t="s">
         <v>231</v>
-      </c>
-      <c r="R18" s="3" t="s">
-        <v>232</v>
       </c>
       <c r="S18" s="3" t="s">
         <v>61</v>
@@ -3427,24 +3467,24 @@
         <v>78</v>
       </c>
     </row>
-    <row r="19" spans="1:20" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:21" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>233</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="C19" s="3" t="s">
         <v>234</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="D19" s="3" t="s">
         <v>235</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="E19" s="3" t="s">
         <v>236</v>
       </c>
-      <c r="E19" s="3" t="s">
+      <c r="F19" s="3" t="s">
         <v>237</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>238</v>
       </c>
       <c r="G19" s="3" t="s">
         <v>49</v>
@@ -3453,34 +3493,34 @@
         <v>67</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="J19" s="3" t="s">
         <v>124</v>
       </c>
       <c r="K19" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="L19" s="3" t="s">
         <v>240</v>
-      </c>
-      <c r="L19" s="3" t="s">
-        <v>241</v>
       </c>
       <c r="M19" s="3" t="s">
         <v>164</v>
       </c>
       <c r="N19" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="O19" s="3" t="s">
         <v>242</v>
       </c>
-      <c r="O19" s="3" t="s">
+      <c r="P19" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q19" s="3" t="s">
         <v>243</v>
       </c>
-      <c r="P19" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q19" s="3" t="s">
-        <v>244</v>
-      </c>
       <c r="R19" s="3" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="S19" s="3" t="s">
         <v>61</v>
@@ -3489,24 +3529,24 @@
         <v>78</v>
       </c>
     </row>
-    <row r="20" spans="1:20" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:21" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="B20" s="3" t="s">
         <v>245</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="C20" s="3" t="s">
         <v>246</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="D20" s="3" t="s">
         <v>247</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="E20" s="3" t="s">
         <v>248</v>
       </c>
-      <c r="E20" s="3" t="s">
+      <c r="F20" s="3" t="s">
         <v>249</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>250</v>
       </c>
       <c r="G20" s="3" t="s">
         <v>49</v>
@@ -3515,34 +3555,34 @@
         <v>67</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="J20" s="3" t="s">
         <v>69</v>
       </c>
       <c r="K20" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="L20" s="3" t="s">
         <v>252</v>
-      </c>
-      <c r="L20" s="3" t="s">
-        <v>253</v>
       </c>
       <c r="M20" s="3" t="s">
         <v>112</v>
       </c>
       <c r="N20" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="O20" s="3" t="s">
         <v>254</v>
       </c>
-      <c r="O20" s="3" t="s">
+      <c r="P20" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q20" s="3" t="s">
         <v>255</v>
       </c>
-      <c r="P20" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q20" s="3" t="s">
+      <c r="R20" s="3" t="s">
         <v>256</v>
-      </c>
-      <c r="R20" s="3" t="s">
-        <v>257</v>
       </c>
       <c r="S20" s="3" t="s">
         <v>61</v>
@@ -3551,24 +3591,24 @@
         <v>62</v>
       </c>
     </row>
-    <row r="21" spans="1:20" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:21" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="B21" s="3" t="s">
         <v>258</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="C21" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="D21" s="3" t="s">
         <v>259</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>247</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>260</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>47</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G21" s="3" t="s">
         <v>122</v>
@@ -3577,34 +3617,34 @@
         <v>50</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="J21" s="3" t="s">
         <v>69</v>
       </c>
       <c r="K21" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="L21" s="3" t="s">
         <v>263</v>
-      </c>
-      <c r="L21" s="3" t="s">
-        <v>264</v>
       </c>
       <c r="M21" s="3" t="s">
         <v>85</v>
       </c>
       <c r="N21" s="3" t="s">
+        <v>264</v>
+      </c>
+      <c r="O21" s="3" t="s">
         <v>265</v>
       </c>
-      <c r="O21" s="3" t="s">
+      <c r="P21" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q21" s="3" t="s">
         <v>266</v>
       </c>
-      <c r="P21" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q21" s="3" t="s">
-        <v>267</v>
-      </c>
       <c r="R21" s="3" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="S21" s="3" t="s">
         <v>141</v>
@@ -3613,24 +3653,24 @@
         <v>62</v>
       </c>
     </row>
-    <row r="22" spans="1:20" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:21" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
+        <v>267</v>
+      </c>
+      <c r="B22" s="3" t="s">
         <v>268</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="C22" s="3" t="s">
         <v>269</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="D22" s="3" t="s">
         <v>270</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="E22" s="3" t="s">
         <v>271</v>
       </c>
-      <c r="E22" s="3" t="s">
+      <c r="F22" s="3" t="s">
         <v>272</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>273</v>
       </c>
       <c r="G22" s="3" t="s">
         <v>49</v>
@@ -3639,54 +3679,54 @@
         <v>67</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="J22" s="3" t="s">
         <v>69</v>
       </c>
       <c r="K22" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="L22" s="3" t="s">
         <v>275</v>
       </c>
-      <c r="L22" s="3" t="s">
+      <c r="M22" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="M22" s="3" t="s">
+      <c r="N22" s="3" t="s">
         <v>277</v>
       </c>
-      <c r="N22" s="3" t="s">
+      <c r="O22" s="3" t="s">
         <v>278</v>
       </c>
-      <c r="O22" s="3" t="s">
+      <c r="P22" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q22" s="3" t="s">
         <v>279</v>
       </c>
-      <c r="P22" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q22" s="3" t="s">
+      <c r="R22" s="3" t="s">
         <v>280</v>
-      </c>
-      <c r="R22" s="3" t="s">
-        <v>281</v>
       </c>
       <c r="S22" s="3" t="s">
         <v>61</v>
       </c>
       <c r="T22" s="3" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="23" spans="1:21" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="3" t="s">
         <v>282</v>
       </c>
-    </row>
-    <row r="23" spans="1:20" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="3" t="s">
+      <c r="B23" s="3" t="s">
         <v>283</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="C23" s="3" t="s">
         <v>284</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="D23" s="3" t="s">
         <v>285</v>
-      </c>
-      <c r="D23" s="3" t="s">
-        <v>286</v>
       </c>
       <c r="E23" s="3" t="s">
         <v>94</v>
@@ -3701,13 +3741,13 @@
         <v>50</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="J23" s="3" t="s">
         <v>52</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="L23" s="3" t="s">
         <v>137</v>
@@ -3716,16 +3756,16 @@
         <v>85</v>
       </c>
       <c r="N23" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="O23" s="3" t="s">
         <v>289</v>
       </c>
-      <c r="O23" s="3" t="s">
+      <c r="P23" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q23" s="3" t="s">
         <v>290</v>
-      </c>
-      <c r="P23" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q23" s="3" t="s">
-        <v>291</v>
       </c>
       <c r="R23" s="3" t="s">
         <v>89</v>
@@ -3737,24 +3777,24 @@
         <v>62</v>
       </c>
     </row>
-    <row r="24" spans="1:20" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:21" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="B24" s="3" t="s">
         <v>292</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="C24" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="D24" s="3" t="s">
         <v>293</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>285</v>
-      </c>
-      <c r="D24" s="3" t="s">
-        <v>294</v>
       </c>
       <c r="E24" s="3" t="s">
         <v>94</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="G24" s="3" t="s">
         <v>122</v>
@@ -3763,31 +3803,31 @@
         <v>67</v>
       </c>
       <c r="I24" s="3" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="J24" s="3" t="s">
         <v>124</v>
       </c>
       <c r="K24" s="3" t="s">
+        <v>296</v>
+      </c>
+      <c r="L24" s="3" t="s">
         <v>297</v>
-      </c>
-      <c r="L24" s="3" t="s">
-        <v>298</v>
       </c>
       <c r="M24" s="3" t="s">
         <v>112</v>
       </c>
       <c r="N24" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="O24" s="3" t="s">
         <v>299</v>
       </c>
-      <c r="O24" s="3" t="s">
+      <c r="P24" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q24" s="3" t="s">
         <v>300</v>
-      </c>
-      <c r="P24" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q24" s="3" t="s">
-        <v>301</v>
       </c>
       <c r="R24" s="3" t="s">
         <v>89</v>
@@ -3799,24 +3839,24 @@
         <v>62</v>
       </c>
     </row>
-    <row r="25" spans="1:20" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:21" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
+        <v>301</v>
+      </c>
+      <c r="B25" s="3" t="s">
         <v>302</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="C25" s="3" t="s">
         <v>303</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="D25" s="3" t="s">
         <v>304</v>
       </c>
-      <c r="D25" s="3" t="s">
+      <c r="E25" s="3" t="s">
         <v>305</v>
       </c>
-      <c r="E25" s="3" t="s">
+      <c r="F25" s="3" t="s">
         <v>306</v>
-      </c>
-      <c r="F25" s="3" t="s">
-        <v>307</v>
       </c>
       <c r="G25" s="3" t="s">
         <v>122</v>
@@ -3825,60 +3865,60 @@
         <v>67</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="J25" s="3" t="s">
         <v>124</v>
       </c>
       <c r="K25" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="L25" s="3" t="s">
         <v>309</v>
-      </c>
-      <c r="L25" s="3" t="s">
-        <v>310</v>
       </c>
       <c r="M25" s="3" t="s">
         <v>112</v>
       </c>
       <c r="N25" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="O25" s="3" t="s">
         <v>311</v>
       </c>
-      <c r="O25" s="3" t="s">
+      <c r="P25" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q25" s="3" t="s">
         <v>312</v>
       </c>
-      <c r="P25" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q25" s="3" t="s">
+      <c r="R25" s="3" t="s">
         <v>313</v>
       </c>
-      <c r="R25" s="3" t="s">
+      <c r="S25" s="3" t="s">
         <v>314</v>
       </c>
-      <c r="S25" s="3" t="s">
+      <c r="T25" s="3" t="s">
         <v>315</v>
       </c>
-      <c r="T25" s="3" t="s">
+    </row>
+    <row r="26" spans="1:21" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="3" t="s">
         <v>316</v>
       </c>
-    </row>
-    <row r="26" spans="1:20" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="3" t="s">
+      <c r="B26" s="3" t="s">
         <v>317</v>
       </c>
-      <c r="B26" s="3" t="s">
+      <c r="C26" s="3" t="s">
         <v>318</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="D26" s="3" t="s">
         <v>319</v>
       </c>
-      <c r="D26" s="3" t="s">
+      <c r="E26" s="3" t="s">
         <v>320</v>
       </c>
-      <c r="E26" s="3" t="s">
+      <c r="F26" s="3" t="s">
         <v>321</v>
-      </c>
-      <c r="F26" s="3" t="s">
-        <v>322</v>
       </c>
       <c r="G26" s="3" t="s">
         <v>49</v>
@@ -3887,34 +3927,34 @@
         <v>67</v>
       </c>
       <c r="I26" s="3" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="J26" s="3" t="s">
         <v>124</v>
       </c>
       <c r="K26" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="L26" s="3" t="s">
         <v>324</v>
-      </c>
-      <c r="L26" s="3" t="s">
-        <v>325</v>
       </c>
       <c r="M26" s="3" t="s">
         <v>85</v>
       </c>
       <c r="N26" s="3" t="s">
+        <v>325</v>
+      </c>
+      <c r="O26" s="3" t="s">
         <v>326</v>
       </c>
-      <c r="O26" s="3" t="s">
+      <c r="P26" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q26" s="3" t="s">
         <v>327</v>
       </c>
-      <c r="P26" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q26" s="3" t="s">
+      <c r="R26" s="3" t="s">
         <v>328</v>
-      </c>
-      <c r="R26" s="3" t="s">
-        <v>329</v>
       </c>
       <c r="S26" s="3" t="s">
         <v>141</v>
@@ -3923,24 +3963,24 @@
         <v>62</v>
       </c>
     </row>
-    <row r="27" spans="1:20" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:21" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="B27" s="3" t="s">
         <v>330</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="C27" s="3" t="s">
         <v>331</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="D27" s="3" t="s">
         <v>332</v>
       </c>
-      <c r="D27" s="3" t="s">
+      <c r="E27" s="3" t="s">
         <v>333</v>
       </c>
-      <c r="E27" s="3" t="s">
+      <c r="F27" s="3" t="s">
         <v>334</v>
-      </c>
-      <c r="F27" s="3" t="s">
-        <v>335</v>
       </c>
       <c r="G27" s="3" t="s">
         <v>49</v>
@@ -3949,34 +3989,34 @@
         <v>67</v>
       </c>
       <c r="I27" s="3" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="J27" s="3" t="s">
         <v>124</v>
       </c>
       <c r="K27" s="3" t="s">
+        <v>336</v>
+      </c>
+      <c r="L27" s="3" t="s">
         <v>337</v>
       </c>
-      <c r="L27" s="3" t="s">
+      <c r="M27" s="3" t="s">
         <v>338</v>
       </c>
-      <c r="M27" s="3" t="s">
+      <c r="N27" s="3" t="s">
         <v>339</v>
       </c>
-      <c r="N27" s="3" t="s">
+      <c r="O27" s="3" t="s">
         <v>340</v>
       </c>
-      <c r="O27" s="3" t="s">
+      <c r="P27" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q27" s="3" t="s">
         <v>341</v>
       </c>
-      <c r="P27" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q27" s="3" t="s">
+      <c r="R27" s="3" t="s">
         <v>342</v>
-      </c>
-      <c r="R27" s="3" t="s">
-        <v>343</v>
       </c>
       <c r="S27" s="3" t="s">
         <v>61</v>
@@ -3985,24 +4025,24 @@
         <v>62</v>
       </c>
     </row>
-    <row r="28" spans="1:20" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:21" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="B28" s="3" t="s">
         <v>344</v>
       </c>
-      <c r="B28" s="3" t="s">
+      <c r="C28" s="3" t="s">
         <v>345</v>
       </c>
-      <c r="C28" s="3" t="s">
+      <c r="D28" s="3" t="s">
         <v>346</v>
       </c>
-      <c r="D28" s="3" t="s">
+      <c r="E28" s="3" t="s">
         <v>347</v>
       </c>
-      <c r="E28" s="3" t="s">
+      <c r="F28" s="3" t="s">
         <v>348</v>
-      </c>
-      <c r="F28" s="3" t="s">
-        <v>349</v>
       </c>
       <c r="G28" s="3" t="s">
         <v>49</v>
@@ -4011,34 +4051,34 @@
         <v>67</v>
       </c>
       <c r="I28" s="3" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="J28" s="3" t="s">
         <v>124</v>
       </c>
       <c r="K28" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="L28" s="3" t="s">
         <v>351</v>
-      </c>
-      <c r="L28" s="3" t="s">
-        <v>352</v>
       </c>
       <c r="M28" s="3" t="s">
         <v>85</v>
       </c>
       <c r="N28" s="3" t="s">
+        <v>352</v>
+      </c>
+      <c r="O28" s="3" t="s">
         <v>353</v>
       </c>
-      <c r="O28" s="3" t="s">
+      <c r="P28" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q28" s="3" t="s">
         <v>354</v>
       </c>
-      <c r="P28" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q28" s="3" t="s">
+      <c r="R28" s="3" t="s">
         <v>355</v>
-      </c>
-      <c r="R28" s="3" t="s">
-        <v>356</v>
       </c>
       <c r="S28" s="3" t="s">
         <v>61</v>
@@ -4047,24 +4087,24 @@
         <v>62</v>
       </c>
     </row>
-    <row r="29" spans="1:20" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:21" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
+        <v>356</v>
+      </c>
+      <c r="B29" s="3" t="s">
         <v>357</v>
       </c>
-      <c r="B29" s="3" t="s">
+      <c r="C29" s="3" t="s">
         <v>358</v>
       </c>
-      <c r="C29" s="3" t="s">
+      <c r="D29" s="3" t="s">
         <v>359</v>
       </c>
-      <c r="D29" s="3" t="s">
+      <c r="E29" s="3" t="s">
+        <v>347</v>
+      </c>
+      <c r="F29" s="3" t="s">
         <v>360</v>
-      </c>
-      <c r="E29" s="3" t="s">
-        <v>348</v>
-      </c>
-      <c r="F29" s="3" t="s">
-        <v>361</v>
       </c>
       <c r="G29" s="3" t="s">
         <v>122</v>
@@ -4073,34 +4113,34 @@
         <v>67</v>
       </c>
       <c r="I29" s="3" t="s">
+        <v>361</v>
+      </c>
+      <c r="J29" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="K29" s="3" t="s">
         <v>362</v>
       </c>
-      <c r="J29" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="K29" s="3" t="s">
+      <c r="L29" s="3" t="s">
         <v>363</v>
       </c>
-      <c r="L29" s="3" t="s">
+      <c r="M29" s="3" t="s">
         <v>364</v>
       </c>
-      <c r="M29" s="3" t="s">
+      <c r="N29" s="3" t="s">
         <v>365</v>
       </c>
-      <c r="N29" s="3" t="s">
+      <c r="O29" s="3" t="s">
         <v>366</v>
       </c>
-      <c r="O29" s="3" t="s">
+      <c r="P29" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q29" s="3" t="s">
         <v>367</v>
       </c>
-      <c r="P29" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q29" s="3" t="s">
+      <c r="R29" s="3" t="s">
         <v>368</v>
-      </c>
-      <c r="R29" s="3" t="s">
-        <v>369</v>
       </c>
       <c r="S29" s="3" t="s">
         <v>77</v>
@@ -4109,24 +4149,24 @@
         <v>62</v>
       </c>
     </row>
-    <row r="30" spans="1:20" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:21" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
+        <v>369</v>
+      </c>
+      <c r="B30" s="3" t="s">
         <v>370</v>
       </c>
-      <c r="B30" s="3" t="s">
+      <c r="C30" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="D30" s="3" t="s">
         <v>371</v>
       </c>
-      <c r="C30" s="3" t="s">
-        <v>314</v>
-      </c>
-      <c r="D30" s="3" t="s">
+      <c r="E30" s="3" t="s">
+        <v>347</v>
+      </c>
+      <c r="F30" s="3" t="s">
         <v>372</v>
-      </c>
-      <c r="E30" s="3" t="s">
-        <v>348</v>
-      </c>
-      <c r="F30" s="3" t="s">
-        <v>373</v>
       </c>
       <c r="G30" s="3" t="s">
         <v>49</v>
@@ -4135,34 +4175,34 @@
         <v>67</v>
       </c>
       <c r="I30" s="3" t="s">
+        <v>373</v>
+      </c>
+      <c r="J30" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="K30" s="3" t="s">
         <v>374</v>
       </c>
-      <c r="J30" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="K30" s="3" t="s">
+      <c r="L30" s="3" t="s">
         <v>375</v>
       </c>
-      <c r="L30" s="3" t="s">
+      <c r="M30" s="3" t="s">
+        <v>364</v>
+      </c>
+      <c r="N30" s="3" t="s">
         <v>376</v>
       </c>
-      <c r="M30" s="3" t="s">
-        <v>365</v>
-      </c>
-      <c r="N30" s="3" t="s">
+      <c r="O30" s="3" t="s">
         <v>377</v>
       </c>
-      <c r="O30" s="3" t="s">
+      <c r="P30" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q30" s="3" t="s">
         <v>378</v>
       </c>
-      <c r="P30" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q30" s="3" t="s">
+      <c r="R30" s="3" t="s">
         <v>379</v>
-      </c>
-      <c r="R30" s="3" t="s">
-        <v>380</v>
       </c>
       <c r="S30" s="3" t="s">
         <v>77</v>
@@ -4171,24 +4211,24 @@
         <v>181</v>
       </c>
     </row>
-    <row r="31" spans="1:20" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:21" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="3" t="s">
+        <v>380</v>
+      </c>
+      <c r="B31" s="3" t="s">
         <v>381</v>
       </c>
-      <c r="B31" s="3" t="s">
+      <c r="C31" s="3" t="s">
         <v>382</v>
       </c>
-      <c r="C31" s="3" t="s">
+      <c r="D31" s="3" t="s">
         <v>383</v>
       </c>
-      <c r="D31" s="3" t="s">
+      <c r="E31" s="3" t="s">
         <v>384</v>
       </c>
-      <c r="E31" s="3" t="s">
+      <c r="F31" s="3" t="s">
         <v>385</v>
-      </c>
-      <c r="F31" s="3" t="s">
-        <v>386</v>
       </c>
       <c r="G31" s="3" t="s">
         <v>122</v>
@@ -4197,34 +4237,34 @@
         <v>67</v>
       </c>
       <c r="I31" s="3" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="J31" s="3" t="s">
         <v>174</v>
       </c>
       <c r="K31" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="L31" s="3" t="s">
         <v>388</v>
-      </c>
-      <c r="L31" s="3" t="s">
-        <v>389</v>
       </c>
       <c r="M31" s="3" t="s">
         <v>164</v>
       </c>
       <c r="N31" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="O31" s="3" t="s">
         <v>390</v>
       </c>
-      <c r="O31" s="3" t="s">
+      <c r="P31" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q31" s="3" t="s">
         <v>391</v>
       </c>
-      <c r="P31" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q31" s="3" t="s">
+      <c r="R31" s="3" t="s">
         <v>392</v>
-      </c>
-      <c r="R31" s="3" t="s">
-        <v>393</v>
       </c>
       <c r="S31" s="3" t="s">
         <v>61</v>
@@ -4233,24 +4273,24 @@
         <v>62</v>
       </c>
     </row>
-    <row r="32" spans="1:20" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:21" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="B32" s="3" t="s">
         <v>394</v>
       </c>
-      <c r="B32" s="3" t="s">
+      <c r="C32" s="3" t="s">
         <v>395</v>
       </c>
-      <c r="C32" s="3" t="s">
+      <c r="D32" s="3" t="s">
         <v>396</v>
-      </c>
-      <c r="D32" s="3" t="s">
-        <v>397</v>
       </c>
       <c r="E32" s="3" t="s">
         <v>121</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="G32" s="3" t="s">
         <v>122</v>
@@ -4259,60 +4299,60 @@
         <v>50</v>
       </c>
       <c r="I32" s="3" t="s">
+        <v>398</v>
+      </c>
+      <c r="J32" s="3" t="s">
         <v>399</v>
       </c>
-      <c r="J32" s="3" t="s">
+      <c r="K32" s="3" t="s">
         <v>400</v>
       </c>
-      <c r="K32" s="3" t="s">
+      <c r="L32" s="3" t="s">
         <v>401</v>
-      </c>
-      <c r="L32" s="3" t="s">
-        <v>402</v>
       </c>
       <c r="M32" s="3" t="s">
         <v>112</v>
       </c>
       <c r="N32" s="3" t="s">
+        <v>402</v>
+      </c>
+      <c r="O32" s="3" t="s">
         <v>403</v>
       </c>
-      <c r="O32" s="3" t="s">
+      <c r="P32" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q32" s="3" t="s">
         <v>404</v>
       </c>
-      <c r="P32" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q32" s="3" t="s">
+      <c r="R32" s="3" t="s">
         <v>405</v>
       </c>
-      <c r="R32" s="3" t="s">
-        <v>406</v>
-      </c>
       <c r="S32" s="3" t="s">
+        <v>314</v>
+      </c>
+      <c r="T32" s="3" t="s">
         <v>315</v>
-      </c>
-      <c r="T32" s="3" t="s">
-        <v>316</v>
       </c>
     </row>
     <row r="33" spans="1:20" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="3" t="s">
+        <v>406</v>
+      </c>
+      <c r="B33" s="3" t="s">
         <v>407</v>
       </c>
-      <c r="B33" s="3" t="s">
+      <c r="C33" s="3" t="s">
         <v>408</v>
       </c>
-      <c r="C33" s="3" t="s">
+      <c r="D33" s="3" t="s">
         <v>409</v>
-      </c>
-      <c r="D33" s="3" t="s">
-        <v>410</v>
       </c>
       <c r="E33" s="3" t="s">
         <v>47</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="G33" s="3" t="s">
         <v>122</v>
@@ -4321,60 +4361,60 @@
         <v>50</v>
       </c>
       <c r="I33" s="3" t="s">
+        <v>411</v>
+      </c>
+      <c r="J33" s="3" t="s">
         <v>412</v>
       </c>
-      <c r="J33" s="3" t="s">
+      <c r="K33" s="3" t="s">
         <v>413</v>
       </c>
-      <c r="K33" s="3" t="s">
+      <c r="L33" s="3" t="s">
         <v>414</v>
-      </c>
-      <c r="L33" s="3" t="s">
-        <v>415</v>
       </c>
       <c r="M33" s="3" t="s">
         <v>85</v>
       </c>
       <c r="N33" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="O33" s="3" t="s">
         <v>416</v>
       </c>
-      <c r="O33" s="3" t="s">
+      <c r="P33" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q33" s="3" t="s">
         <v>417</v>
       </c>
-      <c r="P33" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q33" s="3" t="s">
-        <v>418</v>
-      </c>
       <c r="R33" s="3" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="S33" s="3" t="s">
+        <v>314</v>
+      </c>
+      <c r="T33" s="3" t="s">
         <v>315</v>
-      </c>
-      <c r="T33" s="3" t="s">
-        <v>316</v>
       </c>
     </row>
     <row r="34" spans="1:20" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="3" t="s">
+        <v>418</v>
+      </c>
+      <c r="B34" s="3" t="s">
         <v>419</v>
       </c>
-      <c r="B34" s="3" t="s">
+      <c r="C34" s="3" t="s">
         <v>420</v>
       </c>
-      <c r="C34" s="3" t="s">
+      <c r="D34" s="3" t="s">
         <v>421</v>
       </c>
-      <c r="D34" s="3" t="s">
+      <c r="E34" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="F34" s="3" t="s">
         <v>422</v>
-      </c>
-      <c r="E34" s="3" t="s">
-        <v>306</v>
-      </c>
-      <c r="F34" s="3" t="s">
-        <v>423</v>
       </c>
       <c r="G34" s="3" t="s">
         <v>122</v>
@@ -4383,60 +4423,60 @@
         <v>50</v>
       </c>
       <c r="I34" s="3" t="s">
+        <v>423</v>
+      </c>
+      <c r="J34" s="3" t="s">
         <v>424</v>
       </c>
-      <c r="J34" s="3" t="s">
+      <c r="K34" s="3" t="s">
         <v>425</v>
       </c>
-      <c r="K34" s="3" t="s">
+      <c r="L34" s="3" t="s">
         <v>426</v>
       </c>
-      <c r="L34" s="3" t="s">
+      <c r="M34" s="3" t="s">
         <v>427</v>
       </c>
-      <c r="M34" s="3" t="s">
+      <c r="N34" s="3" t="s">
         <v>428</v>
       </c>
-      <c r="N34" s="3" t="s">
+      <c r="O34" s="3" t="s">
         <v>429</v>
       </c>
-      <c r="O34" s="3" t="s">
+      <c r="P34" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q34" s="3" t="s">
         <v>430</v>
       </c>
-      <c r="P34" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q34" s="3" t="s">
+      <c r="R34" s="3" t="s">
         <v>431</v>
       </c>
-      <c r="R34" s="3" t="s">
+      <c r="S34" s="3" t="s">
         <v>432</v>
       </c>
-      <c r="S34" s="3" t="s">
+      <c r="T34" s="3" t="s">
         <v>433</v>
-      </c>
-      <c r="T34" s="3" t="s">
-        <v>434</v>
       </c>
     </row>
     <row r="35" spans="1:20" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="3" t="s">
+        <v>434</v>
+      </c>
+      <c r="B35" s="3" t="s">
         <v>435</v>
       </c>
-      <c r="B35" s="3" t="s">
+      <c r="C35" s="3" t="s">
         <v>436</v>
       </c>
-      <c r="C35" s="3" t="s">
+      <c r="D35" s="3" t="s">
         <v>437</v>
       </c>
-      <c r="D35" s="3" t="s">
+      <c r="E35" s="3" t="s">
         <v>438</v>
       </c>
-      <c r="E35" s="3" t="s">
+      <c r="F35" s="3" t="s">
         <v>439</v>
-      </c>
-      <c r="F35" s="3" t="s">
-        <v>440</v>
       </c>
       <c r="G35" s="3" t="s">
         <v>122</v>
@@ -4445,34 +4485,34 @@
         <v>67</v>
       </c>
       <c r="I35" s="3" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="J35" s="3" t="s">
         <v>174</v>
       </c>
       <c r="K35" s="3" t="s">
+        <v>441</v>
+      </c>
+      <c r="L35" s="3" t="s">
         <v>442</v>
-      </c>
-      <c r="L35" s="3" t="s">
-        <v>443</v>
       </c>
       <c r="M35" s="3" t="s">
         <v>164</v>
       </c>
       <c r="N35" s="3" t="s">
+        <v>443</v>
+      </c>
+      <c r="O35" s="3" t="s">
         <v>444</v>
       </c>
-      <c r="O35" s="3" t="s">
+      <c r="P35" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q35" s="3" t="s">
         <v>445</v>
       </c>
-      <c r="P35" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q35" s="3" t="s">
+      <c r="R35" s="3" t="s">
         <v>446</v>
-      </c>
-      <c r="R35" s="3" t="s">
-        <v>447</v>
       </c>
       <c r="S35" s="3" t="s">
         <v>141</v>
@@ -4483,22 +4523,22 @@
     </row>
     <row r="36" spans="1:20" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="3" t="s">
+        <v>447</v>
+      </c>
+      <c r="B36" s="3" t="s">
         <v>448</v>
       </c>
-      <c r="B36" s="3" t="s">
+      <c r="C36" s="3" t="s">
         <v>449</v>
       </c>
-      <c r="C36" s="3" t="s">
+      <c r="D36" s="3" t="s">
         <v>450</v>
       </c>
-      <c r="D36" s="3" t="s">
+      <c r="E36" s="3" t="s">
+        <v>347</v>
+      </c>
+      <c r="F36" s="3" t="s">
         <v>451</v>
-      </c>
-      <c r="E36" s="3" t="s">
-        <v>348</v>
-      </c>
-      <c r="F36" s="3" t="s">
-        <v>452</v>
       </c>
       <c r="G36" s="3" t="s">
         <v>122</v>
@@ -4507,37 +4547,37 @@
         <v>67</v>
       </c>
       <c r="I36" s="3" t="s">
+        <v>452</v>
+      </c>
+      <c r="J36" s="3" t="s">
         <v>453</v>
       </c>
-      <c r="J36" s="3" t="s">
+      <c r="K36" s="3" t="s">
         <v>454</v>
       </c>
-      <c r="K36" s="3" t="s">
+      <c r="L36" s="3" t="s">
         <v>455</v>
       </c>
-      <c r="L36" s="3" t="s">
+      <c r="M36" s="3" t="s">
+        <v>364</v>
+      </c>
+      <c r="N36" s="3" t="s">
         <v>456</v>
       </c>
-      <c r="M36" s="3" t="s">
-        <v>365</v>
-      </c>
-      <c r="N36" s="3" t="s">
+      <c r="O36" s="3" t="s">
         <v>457</v>
       </c>
-      <c r="O36" s="3" t="s">
+      <c r="P36" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q36" s="3" t="s">
         <v>458</v>
       </c>
-      <c r="P36" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q36" s="3" t="s">
+      <c r="R36" s="3" t="s">
         <v>459</v>
       </c>
-      <c r="R36" s="3" t="s">
-        <v>460</v>
-      </c>
       <c r="S36" s="3" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="T36" s="3" t="s">
         <v>62</v>
@@ -4545,22 +4585,22 @@
     </row>
     <row r="37" spans="1:20" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="3" t="s">
+        <v>460</v>
+      </c>
+      <c r="B37" s="3" t="s">
         <v>461</v>
       </c>
-      <c r="B37" s="3" t="s">
+      <c r="C37" s="3" t="s">
         <v>462</v>
       </c>
-      <c r="C37" s="3" t="s">
+      <c r="D37" s="3" t="s">
         <v>463</v>
-      </c>
-      <c r="D37" s="3" t="s">
-        <v>464</v>
       </c>
       <c r="E37" s="3" t="s">
         <v>146</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="G37" s="3" t="s">
         <v>122</v>
@@ -4569,60 +4609,60 @@
         <v>50</v>
       </c>
       <c r="I37" s="3" t="s">
+        <v>465</v>
+      </c>
+      <c r="J37" s="3" t="s">
         <v>466</v>
       </c>
-      <c r="J37" s="3" t="s">
+      <c r="K37" s="3" t="s">
         <v>467</v>
       </c>
-      <c r="K37" s="3" t="s">
+      <c r="L37" s="3" t="s">
         <v>468</v>
       </c>
-      <c r="L37" s="3" t="s">
+      <c r="M37" s="3" t="s">
         <v>469</v>
       </c>
-      <c r="M37" s="3" t="s">
+      <c r="N37" s="3" t="s">
         <v>470</v>
       </c>
-      <c r="N37" s="3" t="s">
+      <c r="O37" s="3" t="s">
         <v>471</v>
       </c>
-      <c r="O37" s="3" t="s">
+      <c r="P37" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q37" s="3" t="s">
         <v>472</v>
       </c>
-      <c r="P37" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q37" s="3" t="s">
+      <c r="R37" s="3" t="s">
         <v>473</v>
-      </c>
-      <c r="R37" s="3" t="s">
-        <v>474</v>
       </c>
       <c r="S37" s="3" t="s">
         <v>141</v>
       </c>
       <c r="T37" s="3" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="38" spans="1:20" ht="69.900000000000006" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="3" t="s">
+        <v>474</v>
+      </c>
+      <c r="B38" s="3" t="s">
         <v>475</v>
       </c>
-      <c r="B38" s="3" t="s">
+      <c r="C38" s="3" t="s">
         <v>476</v>
       </c>
-      <c r="C38" s="3" t="s">
+      <c r="D38" s="3" t="s">
         <v>477</v>
       </c>
-      <c r="D38" s="3" t="s">
+      <c r="E38" s="3" t="s">
+        <v>347</v>
+      </c>
+      <c r="F38" s="3" t="s">
         <v>478</v>
-      </c>
-      <c r="E38" s="3" t="s">
-        <v>348</v>
-      </c>
-      <c r="F38" s="3" t="s">
-        <v>479</v>
       </c>
       <c r="G38" s="3" t="s">
         <v>122</v>
@@ -4631,34 +4671,34 @@
         <v>67</v>
       </c>
       <c r="I38" s="3" t="s">
+        <v>479</v>
+      </c>
+      <c r="J38" s="3" t="s">
+        <v>453</v>
+      </c>
+      <c r="K38" s="3" t="s">
         <v>480</v>
       </c>
-      <c r="J38" s="3" t="s">
-        <v>454</v>
-      </c>
-      <c r="K38" s="3" t="s">
+      <c r="L38" s="3" t="s">
         <v>481</v>
       </c>
-      <c r="L38" s="3" t="s">
+      <c r="M38" s="3" t="s">
         <v>482</v>
       </c>
-      <c r="M38" s="3" t="s">
+      <c r="N38" s="3" t="s">
         <v>483</v>
       </c>
-      <c r="N38" s="3" t="s">
+      <c r="O38" s="3" t="s">
         <v>484</v>
       </c>
-      <c r="O38" s="3" t="s">
+      <c r="P38" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q38" s="3" t="s">
         <v>485</v>
       </c>
-      <c r="P38" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q38" s="3" t="s">
+      <c r="R38" s="3" t="s">
         <v>486</v>
-      </c>
-      <c r="R38" s="3" t="s">
-        <v>487</v>
       </c>
       <c r="S38" s="3" t="s">
         <v>61</v>
@@ -4688,12 +4728,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="27.9" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -4718,25 +4758,25 @@
       <c r="Z1" s="4"/>
     </row>
     <row r="2" spans="1:26" ht="33.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="9" t="s">
-        <v>488</v>
-      </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
+      <c r="A2" s="17" t="s">
+        <v>487</v>
+      </c>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
     </row>
     <row r="4" spans="1:26" ht="33.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
+        <v>488</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>489</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>490</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>26</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
     </row>
     <row r="5" spans="1:26" ht="51.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -4744,13 +4784,13 @@
         <v>47</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>491</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>492</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3" t="s">
         <v>493</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>494</v>
       </c>
     </row>
     <row r="6" spans="1:26" ht="51.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -4758,10 +4798,10 @@
         <v>94</v>
       </c>
       <c r="B6" s="3" t="s">
+        <v>494</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>495</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>496</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>69</v>
@@ -4772,41 +4812,41 @@
         <v>186</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>496</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>497</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="3" t="s">
         <v>498</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>499</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="51.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B8" s="3" t="s">
+        <v>499</v>
+      </c>
+      <c r="C8" s="3" t="s">
         <v>500</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>501</v>
-      </c>
       <c r="D8" s="3" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="51.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="B9" s="3" t="s">
+        <v>501</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>502</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="D9" s="3" t="s">
         <v>503</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>504</v>
       </c>
     </row>
   </sheetData>
@@ -4834,12 +4874,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="27.9" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="7" t="s">
-        <v>505</v>
-      </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
+      <c r="A1" s="15" t="s">
+        <v>504</v>
+      </c>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -4864,25 +4904,25 @@
       <c r="Z1" s="4"/>
     </row>
     <row r="2" spans="1:26" ht="33.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="9" t="s">
-        <v>506</v>
-      </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
+      <c r="A2" s="17" t="s">
+        <v>505</v>
+      </c>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
     </row>
     <row r="4" spans="1:26" ht="33.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
+        <v>506</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>507</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="C4" s="1" t="s">
         <v>508</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>509</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>510</v>
       </c>
     </row>
     <row r="5" spans="1:26" ht="51.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -4890,13 +4930,13 @@
         <v>122</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>510</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>511</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3" t="s">
         <v>512</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>513</v>
       </c>
     </row>
     <row r="6" spans="1:26" ht="51.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -4904,13 +4944,13 @@
         <v>49</v>
       </c>
       <c r="B6" s="3" t="s">
+        <v>513</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>514</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="D6" s="3" t="s">
         <v>515</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>516</v>
       </c>
     </row>
     <row r="7" spans="1:26" ht="51.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -4918,13 +4958,13 @@
         <v>50</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>516</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>517</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="3" t="s">
         <v>518</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>519</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="51.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -4932,27 +4972,27 @@
         <v>67</v>
       </c>
       <c r="B8" s="3" t="s">
+        <v>519</v>
+      </c>
+      <c r="C8" s="3" t="s">
         <v>520</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="D8" s="3" t="s">
         <v>521</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>522</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="51.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
+        <v>522</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>523</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="C9" s="3" t="s">
         <v>524</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="D9" s="3" t="s">
         <v>525</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>526</v>
       </c>
     </row>
   </sheetData>
@@ -4980,12 +5020,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="27.9" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="7" t="s">
-        <v>527</v>
-      </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
+      <c r="A1" s="15" t="s">
+        <v>526</v>
+      </c>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -5010,39 +5050,39 @@
       <c r="Z1" s="4"/>
     </row>
     <row r="2" spans="1:26" ht="33.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="9" t="s">
-        <v>528</v>
-      </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
+      <c r="A2" s="17" t="s">
+        <v>527</v>
+      </c>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
     </row>
     <row r="4" spans="1:26" ht="33.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
+        <v>528</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>529</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="C4" s="1" t="s">
         <v>530</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>531</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>532</v>
       </c>
     </row>
     <row r="5" spans="1:26" ht="57.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
+        <v>532</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>533</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>534</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>535</v>
-      </c>
       <c r="D5" s="3" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="6" spans="1:26" ht="57.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -5050,10 +5090,10 @@
         <v>52</v>
       </c>
       <c r="B6" s="3" t="s">
+        <v>535</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>536</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>537</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>62</v>
@@ -5064,27 +5104,27 @@
         <v>124</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>537</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>538</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="3" t="s">
         <v>539</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>540</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="57.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="B8" s="3" t="s">
+        <v>540</v>
+      </c>
+      <c r="C8" s="3" t="s">
         <v>541</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>542</v>
-      </c>
       <c r="D8" s="3" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
   </sheetData>
@@ -5112,12 +5152,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="27.9" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="7" t="s">
-        <v>543</v>
-      </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
+      <c r="A1" s="15" t="s">
+        <v>542</v>
+      </c>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -5142,12 +5182,12 @@
       <c r="Z1" s="4"/>
     </row>
     <row r="2" spans="1:26" ht="33.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="9" t="s">
-        <v>544</v>
-      </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
+      <c r="A2" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
     </row>
     <row r="4" spans="1:26" ht="33.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
@@ -5157,7 +5197,7 @@
         <v>36</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>40</v>
@@ -5168,7 +5208,7 @@
         <v>64</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>69</v>
@@ -5179,16 +5219,16 @@
     </row>
     <row r="6" spans="1:26" ht="51.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>69</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
     </row>
     <row r="7" spans="1:26" ht="51.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -5196,7 +5236,7 @@
         <v>91</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>52</v>
@@ -5210,21 +5250,21 @@
         <v>143</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>52</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="51.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
+        <v>551</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>552</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>553</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>69</v>
@@ -5235,38 +5275,38 @@
     </row>
     <row r="10" spans="1:26" ht="51.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
+        <v>553</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>554</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>555</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>69</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="51.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
+        <v>555</v>
+      </c>
+      <c r="B11" s="3" t="s">
         <v>556</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>557</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>124</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="12" spans="1:26" ht="51.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>124</v>
@@ -5277,30 +5317,30 @@
     </row>
     <row r="13" spans="1:26" ht="51.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>124</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="14" spans="1:26" ht="51.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="B14" s="3" t="s">
+        <v>559</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>453</v>
+      </c>
+      <c r="D14" s="3" t="s">
         <v>560</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>454</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>561</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(matrix): Steward CAP placeholder 補編號 + C1-F traceability
- CAP-NEW (Logging) → CAP-036 (Operational Logging)
- CAP-NEW (Health)  → CAP-024 (Deployment/Health)
- xlsx Tab 2 同步補 CAP-024 / CAP-036 細節
- Auditor: matrix.md C1-F 列 TBD → #13（Issue 已開）

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/compliance/ICS_DMAS_master_capability_matrix.xlsx
+++ b/docs/compliance/ICS_DMAS_master_capability_matrix.xlsx
@@ -258,7 +258,7 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
@@ -328,6 +328,9 @@
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2166,7 +2169,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z39"/>
+  <dimension ref="A1:Z40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="20"/>
   <cols>
     <col width="21" customWidth="1" style="19" min="1" max="1"/>
@@ -4712,7 +4715,9 @@
       </c>
       <c r="K28" s="22" t="inlineStr">
         <is>
-          <t>C3；STRICT_TLS；nginx/step-ca；systemd。</t>
+          <t>C3-B install script; STRICT_TLS; nginx/step-ca; systemd.
+v2.1.0: /health liveness only (L1 partial — Exercise Pro 序列A).
+v2.2.0: /metrics + Prometheus + alert rules (L2 full — GovOps).</t>
         </is>
       </c>
       <c r="L28" s="22" t="inlineStr">
@@ -4742,7 +4747,8 @@
       </c>
       <c r="Q28" s="22" t="inlineStr">
         <is>
-          <t>補 deployment architecture 與 runbook</t>
+          <t>v2.1.0: implement /health basic liveness ({"status":"ok","version":"x.x.x"}).
+v2.2.0: add /metrics Prometheus + alerting.</t>
         </is>
       </c>
       <c r="R28" s="22" t="inlineStr">
@@ -5878,6 +5884,108 @@
         </is>
       </c>
       <c r="T39" t="inlineStr">
+        <is>
+          <t>Internal Only</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="38" t="inlineStr">
+        <is>
+          <t>CAP-036</t>
+        </is>
+      </c>
+      <c r="B40" s="38" t="inlineStr">
+        <is>
+          <t>Operational Logging &amp; Debug</t>
+        </is>
+      </c>
+      <c r="C40" s="38" t="inlineStr">
+        <is>
+          <t>Ops / Reliability</t>
+        </is>
+      </c>
+      <c r="D40" s="38" t="inlineStr">
+        <is>
+          <t>Structured JSON logging (structlog), correlation ID, 8 priority log positions, log persistence to /var/log/ics/, collect_debug.sh one-command debug package.</t>
+        </is>
+      </c>
+      <c r="E40" s="38" t="inlineStr">
+        <is>
+          <t>GP2, GP3, GP4</t>
+        </is>
+      </c>
+      <c r="F40" s="38" t="inlineStr">
+        <is>
+          <t>DevOps, 現場維運人員</t>
+        </is>
+      </c>
+      <c r="G40" s="38" t="inlineStr">
+        <is>
+          <t>L0</t>
+        </is>
+      </c>
+      <c r="H40" s="38" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="I40" s="38" t="inlineStr">
+        <is>
+          <t>ERROR log 持久化；collect_debug.sh 產出 zip；correlation ID 跨組件追蹤；prod mode 只出 INFO+；8 個優先位置有 log。</t>
+        </is>
+      </c>
+      <c r="J40" s="38" t="inlineStr">
+        <is>
+          <t>Exercise Pro</t>
+        </is>
+      </c>
+      <c r="K40" s="38" t="inlineStr">
+        <is>
+          <t>C1-D; 部署基礎設施，在所有 P0 Security 之前完成</t>
+        </is>
+      </c>
+      <c r="L40" s="38" t="inlineStr">
+        <is>
+          <t>NIST AU-2, AU-3, AU-12, SI-11</t>
+        </is>
+      </c>
+      <c r="M40" s="38" t="inlineStr">
+        <is>
+          <t>Low (log metadata)</t>
+        </is>
+      </c>
+      <c r="N40" s="38" t="inlineStr">
+        <is>
+          <t>PR# (TBD); collect_debug.sh demo; log rotation verify</t>
+        </is>
+      </c>
+      <c r="O40" s="38" t="inlineStr">
+        <is>
+          <t>支援現場問題診斷與事後稽核</t>
+        </is>
+      </c>
+      <c r="P40" s="38" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="Q40" s="38" t="inlineStr">
+        <is>
+          <t>序列 A — 部署基礎設施，最優先</t>
+        </is>
+      </c>
+      <c r="R40" s="38" t="inlineStr">
+        <is>
+          <t>DevOps / Backend</t>
+        </is>
+      </c>
+      <c r="S40" s="38" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="T40" s="38" t="inlineStr">
         <is>
           <t>Internal Only</t>
         </is>
@@ -5946,7 +6054,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="34" customHeight="1">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -6337,7 +6444,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="34" customHeight="1">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -7088,7 +7194,7 @@
       </c>
       <c r="D7" s="30" t="inlineStr">
         <is>
-          <t>CAP-NEW (Logging)</t>
+          <t>CAP-036 (Operational Logging)</t>
         </is>
       </c>
       <c r="E7" s="30" t="inlineStr">
@@ -7130,7 +7236,7 @@
       </c>
       <c r="D8" s="30" t="inlineStr">
         <is>
-          <t>CAP-024 (Deployment/Health)</t>
+          <t>CAP-024 (Deployment/Health) — partial L1 (/health only; full L2 in v2.2.0)</t>
         </is>
       </c>
       <c r="E8" s="30" t="inlineStr">

</xml_diff>